<commit_message>
Import DONE! Tests grønne!
</commit_message>
<xml_diff>
--- a/CollectaMundo.Tests/TestResources/ImportTest2.xlsx
+++ b/CollectaMundo.Tests/TestResources/ImportTest2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\code\CollectaMundo.Tests\TestResources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{A5ED746B-064A-44FD-B5EC-CD4D64B08518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5CE8187-8529-4231-9A8E-C614D3758D19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="5390" windowWidth="19420" windowHeight="12220" xr2:uid="{19679B59-590C-43DF-AF72-4BC22B219E98}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="38700" windowHeight="15225" xr2:uid="{19679B59-590C-43DF-AF72-4BC22B219E98}"/>
   </bookViews>
   <sheets>
     <sheet name="ImportTest2" sheetId="1" r:id="rId1"/>
@@ -1159,7 +1159,7 @@
         <v>1</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C5" t="s">
         <v>17</v>

</xml_diff>